<commit_message>
comparisons for updated data figs
</commit_message>
<xml_diff>
--- a/output/ATable-group-char-control.xlsx
+++ b/output/ATable-group-char-control.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T12"/>
+  <dimension ref="A1:U12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -362,95 +362,100 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>cat</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>NumberofHotels</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>share_rooms</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Rooms</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>ShareRestaurant</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Stars</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>YearBuilt</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>YearLastRenovated</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>TaxesPaid</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>ADR</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>RevPAR</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Occupancy</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Demand</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>MedianIncome</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>shareWhite</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>shareHisp</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>shareBlack</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>shareAsian</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>plot_label</t>
         </is>
@@ -462,61 +467,66 @@
           <t>C11</t>
         </is>
       </c>
-      <c r="B2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>control-othercity</t>
+        </is>
+      </c>
+      <c r="C2">
         <v>12</v>
       </c>
-      <c r="C2">
-        <v>8117800</v>
-      </c>
       <c r="D2">
+        <v>9653600</v>
+      </c>
+      <c r="E2">
         <v>183</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>57</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>3.5</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>2002</v>
       </c>
-      <c r="H2">
-        <v>2017</v>
-      </c>
       <c r="I2">
-        <v>439</v>
+        <v>2016</v>
       </c>
       <c r="J2">
-        <v>155.76</v>
+        <v>566</v>
       </c>
       <c r="K2">
-        <v>130.1</v>
+        <v>156.99</v>
       </c>
       <c r="L2">
-        <v>9.1</v>
+        <v>131.21</v>
       </c>
       <c r="M2">
-        <v>83.40000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="N2">
-        <v>58429</v>
+        <v>83.5</v>
       </c>
       <c r="O2">
+        <v>58445</v>
+      </c>
+      <c r="P2">
         <v>173</v>
       </c>
-      <c r="P2">
+      <c r="Q2">
         <v>53.1</v>
       </c>
-      <c r="Q2">
+      <c r="R2">
         <v>20.6</v>
       </c>
-      <c r="R2">
+      <c r="S2">
         <v>3.5</v>
       </c>
-      <c r="S2">
+      <c r="T2">
         <v>14.2</v>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>Airport - Upscale - Large</t>
         </is>
@@ -528,61 +538,66 @@
           <t>C01</t>
         </is>
       </c>
-      <c r="B3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>control-union</t>
+        </is>
+      </c>
+      <c r="C3">
         <v>9</v>
       </c>
-      <c r="C3">
-        <v>19846800</v>
-      </c>
       <c r="D3">
+        <v>23597200</v>
+      </c>
+      <c r="E3">
         <v>596</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>100</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>3.9</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>1980</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>2021</v>
       </c>
-      <c r="I3">
-        <v>1062</v>
-      </c>
       <c r="J3">
-        <v>157.14</v>
+        <v>1099</v>
       </c>
       <c r="K3">
-        <v>122.34</v>
+        <v>159.3</v>
       </c>
       <c r="L3">
+        <v>124.19</v>
+      </c>
+      <c r="M3">
+        <v>21.3</v>
+      </c>
+      <c r="N3">
+        <v>77.8</v>
+      </c>
+      <c r="O3">
+        <v>133257</v>
+      </c>
+      <c r="P3">
+        <v>103</v>
+      </c>
+      <c r="Q3">
         <v>21</v>
       </c>
-      <c r="M3">
-        <v>77.7</v>
-      </c>
-      <c r="N3">
-        <v>133162</v>
-      </c>
-      <c r="O3">
-        <v>103</v>
-      </c>
-      <c r="P3">
-        <v>21</v>
-      </c>
-      <c r="Q3">
+      <c r="R3">
         <v>49.3</v>
       </c>
-      <c r="R3">
+      <c r="S3">
         <v>14.9</v>
       </c>
-      <c r="S3">
+      <c r="T3">
         <v>9.199999999999999</v>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>Airport - Upscale - Mega</t>
         </is>
@@ -594,61 +609,66 @@
           <t>C03</t>
         </is>
       </c>
-      <c r="B4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>control-union</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>6</v>
+      </c>
+      <c r="D4">
+        <v>4980800</v>
+      </c>
+      <c r="E4">
+        <v>189</v>
+      </c>
+      <c r="F4">
+        <v>100</v>
+      </c>
+      <c r="G4">
+        <v>4</v>
+      </c>
+      <c r="H4">
+        <v>1965</v>
+      </c>
+      <c r="I4">
+        <v>2019</v>
+      </c>
+      <c r="J4">
+        <v>946</v>
+      </c>
+      <c r="K4">
+        <v>274.63</v>
+      </c>
+      <c r="L4">
+        <v>193.89</v>
+      </c>
+      <c r="M4">
         <v>7</v>
       </c>
-      <c r="C4">
-        <v>4595400</v>
-      </c>
-      <c r="D4">
-        <v>177</v>
-      </c>
-      <c r="E4">
-        <v>91.09999999999999</v>
-      </c>
-      <c r="F4">
-        <v>3.9</v>
-      </c>
-      <c r="G4">
-        <v>1961</v>
-      </c>
-      <c r="H4">
-        <v>2019</v>
-      </c>
-      <c r="I4">
-        <v>863</v>
-      </c>
-      <c r="J4">
-        <v>267.99</v>
-      </c>
-      <c r="K4">
-        <v>188.27</v>
-      </c>
-      <c r="L4">
-        <v>6.8</v>
-      </c>
-      <c r="M4">
-        <v>70.09999999999999</v>
-      </c>
       <c r="N4">
-        <v>25337</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="O4">
-        <v>85</v>
+        <v>25447</v>
       </c>
       <c r="P4">
-        <v>19</v>
+        <v>84</v>
       </c>
       <c r="Q4">
-        <v>46.5</v>
+        <v>18.2</v>
       </c>
       <c r="R4">
-        <v>10.7</v>
+        <v>48.5</v>
       </c>
       <c r="S4">
-        <v>19.3</v>
-      </c>
-      <c r="T4" t="inlineStr">
+        <v>10.3</v>
+      </c>
+      <c r="T4">
+        <v>18.7</v>
+      </c>
+      <c r="U4" t="inlineStr">
         <is>
           <t>Downtown (CBD) - Luxury - Large</t>
         </is>
@@ -660,61 +680,66 @@
           <t>C06</t>
         </is>
       </c>
-      <c r="B5">
-        <v>21</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>control-small</t>
+        </is>
       </c>
       <c r="C5">
-        <v>3685200</v>
+        <v>20</v>
       </c>
       <c r="D5">
-        <v>47</v>
+        <v>4241600</v>
       </c>
       <c r="E5">
-        <v>44.7</v>
+        <v>48</v>
       </c>
       <c r="F5">
-        <v>2.5</v>
+        <v>41.3</v>
       </c>
       <c r="G5">
-        <v>1969</v>
+        <v>2.6</v>
       </c>
       <c r="H5">
-        <v>2005</v>
+        <v>1972</v>
       </c>
       <c r="I5">
-        <v>62</v>
+        <v>2018</v>
       </c>
       <c r="J5">
-        <v>141.95</v>
+        <v>68</v>
       </c>
       <c r="K5">
-        <v>98.58</v>
+        <v>143.3</v>
       </c>
       <c r="L5">
+        <v>99.06999999999999</v>
+      </c>
+      <c r="M5">
         <v>2.9</v>
       </c>
-      <c r="M5">
-        <v>69.2</v>
-      </c>
       <c r="N5">
-        <v>20640</v>
+        <v>69</v>
       </c>
       <c r="O5">
-        <v>83</v>
+        <v>19874</v>
       </c>
       <c r="P5">
-        <v>11</v>
+        <v>82</v>
       </c>
       <c r="Q5">
-        <v>54.3</v>
+        <v>10.4</v>
       </c>
       <c r="R5">
-        <v>11.6</v>
+        <v>55.6</v>
       </c>
       <c r="S5">
-        <v>19.6</v>
-      </c>
-      <c r="T5" t="inlineStr">
+        <v>11.3</v>
+      </c>
+      <c r="T5">
+        <v>19.4</v>
+      </c>
+      <c r="U5" t="inlineStr">
         <is>
           <t>Downtown (CBD) - Luxury - Small</t>
         </is>
@@ -726,61 +751,66 @@
           <t>C04</t>
         </is>
       </c>
-      <c r="B6">
-        <v>12</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>control-union</t>
+        </is>
       </c>
       <c r="C6">
-        <v>24471800</v>
+        <v>11</v>
       </c>
       <c r="D6">
-        <v>551</v>
+        <v>28617600</v>
       </c>
       <c r="E6">
-        <v>93</v>
+        <v>591</v>
       </c>
       <c r="F6">
+        <v>100</v>
+      </c>
+      <c r="G6">
         <v>4</v>
       </c>
-      <c r="G6">
-        <v>1988</v>
-      </c>
       <c r="H6">
-        <v>2018</v>
+        <v>1989</v>
       </c>
       <c r="I6">
-        <v>829</v>
+        <v>2017</v>
       </c>
       <c r="J6">
-        <v>226.66</v>
+        <v>583</v>
       </c>
       <c r="K6">
-        <v>155.05</v>
+        <v>228.84</v>
       </c>
       <c r="L6">
-        <v>31.9</v>
+        <v>158.61</v>
       </c>
       <c r="M6">
-        <v>68.3</v>
+        <v>32.7</v>
       </c>
       <c r="N6">
-        <v>140705</v>
+        <v>69.2</v>
       </c>
       <c r="O6">
+        <v>142623</v>
+      </c>
+      <c r="P6">
         <v>90</v>
       </c>
-      <c r="P6">
-        <v>19.7</v>
-      </c>
       <c r="Q6">
-        <v>42</v>
+        <v>19.5</v>
       </c>
       <c r="R6">
-        <v>11</v>
+        <v>42.2</v>
       </c>
       <c r="S6">
+        <v>10.9</v>
+      </c>
+      <c r="T6">
         <v>22.6</v>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>Downtown (CBD) - Upscale - Mega</t>
         </is>
@@ -789,64 +819,69 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C02</t>
-        </is>
-      </c>
-      <c r="B7">
-        <v>9</v>
+          <t>C07</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>control-othercity</t>
+        </is>
       </c>
       <c r="C7">
-        <v>9738400</v>
+        <v>11</v>
       </c>
       <c r="D7">
-        <v>292</v>
+        <v>8808800</v>
       </c>
       <c r="E7">
-        <v>95.8</v>
+        <v>182</v>
       </c>
       <c r="F7">
-        <v>3.9</v>
+        <v>95.7</v>
       </c>
       <c r="G7">
-        <v>1983</v>
+        <v>4.3</v>
       </c>
       <c r="H7">
-        <v>2015</v>
+        <v>1963</v>
       </c>
       <c r="I7">
-        <v>573</v>
+        <v>2021</v>
       </c>
       <c r="J7">
-        <v>331.34</v>
+        <v>1635</v>
       </c>
       <c r="K7">
-        <v>231.04</v>
+        <v>833.64</v>
       </c>
       <c r="L7">
-        <v>18.6</v>
+        <v>512.84</v>
       </c>
       <c r="M7">
-        <v>69.7</v>
+        <v>33.6</v>
       </c>
       <c r="N7">
-        <v>56113</v>
+        <v>61.3</v>
       </c>
       <c r="O7">
-        <v>125</v>
+        <v>40267</v>
       </c>
       <c r="P7">
-        <v>58.7</v>
+        <v>165</v>
       </c>
       <c r="Q7">
-        <v>16.9</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="R7">
-        <v>5.2</v>
+        <v>7.3</v>
       </c>
       <c r="S7">
-        <v>12.1</v>
-      </c>
-      <c r="T7" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="T7">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="U7" t="inlineStr">
         <is>
           <t>Hollywood/West LA - Luxury - Large</t>
         </is>
@@ -855,64 +890,69 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C07</t>
-        </is>
-      </c>
-      <c r="B8">
-        <v>11</v>
+          <t>C08</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>control-othercity</t>
+        </is>
       </c>
       <c r="C8">
-        <v>7440700</v>
+        <v>14</v>
       </c>
       <c r="D8">
-        <v>183</v>
+        <v>9288400</v>
       </c>
       <c r="E8">
-        <v>95.7</v>
+        <v>151</v>
       </c>
       <c r="F8">
-        <v>4.3</v>
+        <v>95.3</v>
       </c>
       <c r="G8">
-        <v>1963</v>
+        <v>3.9</v>
       </c>
       <c r="H8">
-        <v>2020</v>
+        <v>1979</v>
       </c>
       <c r="I8">
-        <v>1449</v>
+        <v>2018</v>
       </c>
       <c r="J8">
-        <v>814.24</v>
+        <v>1335</v>
       </c>
       <c r="K8">
-        <v>492.41</v>
+        <v>360.22</v>
       </c>
       <c r="L8">
-        <v>32.8</v>
+        <v>256.5</v>
       </c>
       <c r="M8">
-        <v>60.4</v>
+        <v>17.3</v>
       </c>
       <c r="N8">
-        <v>40221</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="O8">
-        <v>165</v>
+        <v>47877</v>
       </c>
       <c r="P8">
-        <v>74.59999999999999</v>
+        <v>141</v>
       </c>
       <c r="Q8">
-        <v>7.3</v>
+        <v>71.2</v>
       </c>
       <c r="R8">
-        <v>2</v>
+        <v>11.6</v>
       </c>
       <c r="S8">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="T8" t="inlineStr">
+        <v>3.2</v>
+      </c>
+      <c r="T8">
+        <v>7.1</v>
+      </c>
+      <c r="U8" t="inlineStr">
         <is>
           <t>Hollywood/West LA - Luxury - Large</t>
         </is>
@@ -921,64 +961,69 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C08</t>
-        </is>
-      </c>
-      <c r="B9">
-        <v>14</v>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>control-othercity</t>
+        </is>
       </c>
       <c r="C9">
-        <v>7810700</v>
+        <v>17</v>
       </c>
       <c r="D9">
-        <v>151</v>
+        <v>12856800</v>
       </c>
       <c r="E9">
-        <v>95.3</v>
+        <v>172</v>
       </c>
       <c r="F9">
-        <v>3.9</v>
+        <v>95.8</v>
       </c>
       <c r="G9">
-        <v>1979</v>
+        <v>4.1</v>
       </c>
       <c r="H9">
-        <v>2018</v>
+        <v>1967</v>
       </c>
       <c r="I9">
-        <v>1125</v>
+        <v>2020</v>
       </c>
       <c r="J9">
-        <v>357.16</v>
+        <v>1077</v>
       </c>
       <c r="K9">
-        <v>251.39</v>
+        <v>424.59</v>
       </c>
       <c r="L9">
-        <v>16.9</v>
+        <v>316.57</v>
       </c>
       <c r="M9">
-        <v>70.3</v>
+        <v>29</v>
       </c>
       <c r="N9">
-        <v>47352</v>
+        <v>74.3</v>
       </c>
       <c r="O9">
-        <v>141</v>
+        <v>67927</v>
       </c>
       <c r="P9">
-        <v>71.2</v>
+        <v>136</v>
       </c>
       <c r="Q9">
-        <v>11.6</v>
+        <v>63.6</v>
       </c>
       <c r="R9">
-        <v>3.2</v>
+        <v>14.7</v>
       </c>
       <c r="S9">
-        <v>7.1</v>
-      </c>
-      <c r="T9" t="inlineStr">
+        <v>4.9</v>
+      </c>
+      <c r="T9">
+        <v>9.1</v>
+      </c>
+      <c r="U9" t="inlineStr">
         <is>
           <t>Hollywood/West LA - Luxury - Large</t>
         </is>
@@ -987,66 +1032,71 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C10</t>
-        </is>
-      </c>
-      <c r="B10">
-        <v>17</v>
+          <t>C02</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>control-union</t>
+        </is>
       </c>
       <c r="C10">
-        <v>10815100</v>
+        <v>8</v>
       </c>
       <c r="D10">
-        <v>172</v>
+        <v>11096800</v>
       </c>
       <c r="E10">
-        <v>93.2</v>
+        <v>315</v>
       </c>
       <c r="F10">
+        <v>100</v>
+      </c>
+      <c r="G10">
         <v>4.1</v>
       </c>
-      <c r="G10">
-        <v>1967</v>
-      </c>
       <c r="H10">
-        <v>2020</v>
+        <v>1986</v>
       </c>
       <c r="I10">
-        <v>958</v>
+        <v>2018</v>
       </c>
       <c r="J10">
-        <v>415.28</v>
+        <v>608</v>
       </c>
       <c r="K10">
-        <v>308.47</v>
+        <v>338.09</v>
       </c>
       <c r="L10">
-        <v>28.1</v>
+        <v>237.27</v>
       </c>
       <c r="M10">
-        <v>74.09999999999999</v>
+        <v>19.1</v>
       </c>
       <c r="N10">
-        <v>67484</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="O10">
-        <v>136</v>
+        <v>56410</v>
       </c>
       <c r="P10">
-        <v>63.6</v>
+        <v>127</v>
       </c>
       <c r="Q10">
-        <v>14.7</v>
+        <v>60.1</v>
       </c>
       <c r="R10">
-        <v>4.9</v>
+        <v>16.5</v>
       </c>
       <c r="S10">
-        <v>9.1</v>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>Hollywood/West LA - Luxury - Large</t>
+        <v>4.8</v>
+      </c>
+      <c r="T10">
+        <v>11.6</v>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Hollywood/West LA - Luxury - Mega</t>
         </is>
       </c>
     </row>
@@ -1056,61 +1106,66 @@
           <t>C05</t>
         </is>
       </c>
-      <c r="B11">
-        <v>24</v>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>control-small</t>
+        </is>
       </c>
       <c r="C11">
-        <v>4240200</v>
+        <v>26</v>
       </c>
       <c r="D11">
+        <v>5478000</v>
+      </c>
+      <c r="E11">
         <v>48</v>
       </c>
-      <c r="E11">
-        <v>17.6</v>
-      </c>
       <c r="F11">
+        <v>20.6</v>
+      </c>
+      <c r="G11">
         <v>2.8</v>
       </c>
-      <c r="G11">
-        <v>1966</v>
-      </c>
       <c r="H11">
-        <v>2020</v>
+        <v>1964</v>
       </c>
       <c r="I11">
-        <v>78</v>
+        <v>2021</v>
       </c>
       <c r="J11">
-        <v>171.92</v>
+        <v>89</v>
       </c>
       <c r="K11">
-        <v>121.35</v>
+        <v>180.58</v>
       </c>
       <c r="L11">
-        <v>4</v>
+        <v>128.51</v>
       </c>
       <c r="M11">
-        <v>70.40000000000001</v>
+        <v>4.7</v>
       </c>
       <c r="N11">
-        <v>23376</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="O11">
+        <v>26046</v>
+      </c>
+      <c r="P11">
         <v>119</v>
       </c>
-      <c r="P11">
-        <v>50.7</v>
-      </c>
       <c r="Q11">
+        <v>51.1</v>
+      </c>
+      <c r="R11">
         <v>23.6</v>
       </c>
-      <c r="R11">
-        <v>4.5</v>
-      </c>
       <c r="S11">
-        <v>14.7</v>
-      </c>
-      <c r="T11" t="inlineStr">
+        <v>4.4</v>
+      </c>
+      <c r="T11">
+        <v>14.4</v>
+      </c>
+      <c r="U11" t="inlineStr">
         <is>
           <t>Hollywood/West LA - Luxury - Small</t>
         </is>
@@ -1122,61 +1177,66 @@
           <t>C09</t>
         </is>
       </c>
-      <c r="B12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>control-othercity</t>
+        </is>
+      </c>
+      <c r="C12">
         <v>6</v>
       </c>
-      <c r="C12">
-        <v>2316200</v>
-      </c>
       <c r="D12">
+        <v>2754400</v>
+      </c>
+      <c r="E12">
         <v>104</v>
       </c>
-      <c r="E12">
+      <c r="F12">
         <v>21.7</v>
       </c>
-      <c r="F12">
+      <c r="G12">
         <v>3.1</v>
       </c>
-      <c r="G12">
+      <c r="H12">
         <v>1984</v>
       </c>
-      <c r="H12">
+      <c r="I12">
         <v>2021</v>
       </c>
-      <c r="I12">
-        <v>359</v>
-      </c>
       <c r="J12">
-        <v>232.29</v>
+        <v>382</v>
       </c>
       <c r="K12">
-        <v>178.58</v>
+        <v>234.09</v>
       </c>
       <c r="L12">
+        <v>182.32</v>
+      </c>
+      <c r="M12">
         <v>3.6</v>
       </c>
-      <c r="M12">
-        <v>76.40000000000001</v>
-      </c>
       <c r="N12">
-        <v>15279</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="O12">
+        <v>15477</v>
+      </c>
+      <c r="P12">
         <v>139</v>
       </c>
-      <c r="P12">
+      <c r="Q12">
         <v>59.1</v>
       </c>
-      <c r="Q12">
+      <c r="R12">
         <v>17.5</v>
       </c>
-      <c r="R12">
+      <c r="S12">
         <v>4.4</v>
       </c>
-      <c r="S12">
+      <c r="T12">
         <v>11.4</v>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>Hollywood/West LA - Midscale - Medium</t>
         </is>

</xml_diff>